<commit_message>
added support page and init files
</commit_message>
<xml_diff>
--- a/testdata/users.xlsx
+++ b/testdata/users.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="16">
   <si>
     <t>username</t>
   </si>
@@ -34,6 +34,36 @@
   </si>
   <si>
     <t>Sriharaye@10</t>
+  </si>
+  <si>
+    <t>type</t>
+  </si>
+  <si>
+    <t>remarks</t>
+  </si>
+  <si>
+    <t>v</t>
+  </si>
+  <si>
+    <t>valid username and valid password</t>
+  </si>
+  <si>
+    <t>iu</t>
+  </si>
+  <si>
+    <t>invalid username and valid password</t>
+  </si>
+  <si>
+    <t>ip</t>
+  </si>
+  <si>
+    <t>invalid password and valid username</t>
+  </si>
+  <si>
+    <t>iup</t>
+  </si>
+  <si>
+    <t>invalid username and invalid password</t>
   </si>
 </sst>
 </file>
@@ -78,7 +108,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
@@ -383,51 +414,81 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="C1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
+      <c r="C2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="2" t="s">
         <v>3</v>
       </c>
+      <c r="C3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="2" t="s">
         <v>5</v>
       </c>
+      <c r="C4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="2" t="s">
         <v>5</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>